<commit_message>
Completo contenido del primer y segundo semestre en el Excel
</commit_message>
<xml_diff>
--- a/estructura_curso.xlsx
+++ b/estructura_curso.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,7 +603,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>[{"nombre": "Presentación de la clase", "url": "https://drive.google.com/..."}]</t>
+          <t>[{"nombre":"Presentación de la clase","url":"https://drive.google.com/..."},{"nombre":"Línea de tiempo interactiva","url":"https://drive.google.com/..."}]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -840,6 +840,641 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>sem1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Semestre I: Fundamentos y Componentes de la Máquina</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Conocer, Tocar, Comprender</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>sem1_clase2</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Clase 2: Componentes del Hardware, Ensamblaje y Normas de Seguridad</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Identificación y manipulación de los componentes físicos de un computador. Normas de seguridad electrostática y técnicas de ensamblaje.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Guía de seguridad y herramientas","url":"https://drive.google.com/..."},{"nombre":"Video: Despiece y ensamblaje","url":"https://www.youtube.com/watch?v=YYYY"}]</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>t2_1</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Demostración en vivo: Despiece de un computador</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>El instructor realiza el despiece completo de un computador mientras explica cada componente y su función.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Imagen/despiece.jpg</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>https://youtu.be/YYYY</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Toma notas de los pasos de seguridad.|Identifica al menos 5 componentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>sem1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Semestre I: Fundamentos y Componentes de la Máquina</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Conocer, Tocar, Comprender</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>sem1_clase2</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Clase 2: Componentes del Hardware, Ensamblaje y Normas de Seguridad</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Identificación y manipulación de los componentes físicos de un computador. Normas de seguridad electrostática y técnicas de ensamblaje.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>t2_2</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Práctica: Ensamblaje con pulsera antiestática</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>En parejas, arman y desarman un computador siguiendo la guía, aplicando normas de seguridad.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Imagen/ensamblaje.jpg</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Usa la pulsera antiestática en todo momento.|Registra cada paso con fotos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>sem1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Semestre I: Fundamentos y Componentes de la Máquina</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Conocer, Tocar, Comprender</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>sem1_clase3</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Clase 3: Sistemas Numéricos y Representación de Datos</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Estudio de los sistemas binario, octal, hexadecimal y su relación con el mundo digital. Conversiones y representación de datos en computadoras.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Tablas de conversión","url":"https://drive.google.com/..."},{"nombre":"Calculadora binaria en línea","url":"https://www.rapidtables.com/convert/number/binary-to-decimal.html"}]</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>t3_1</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Analogía con monedas y billetes</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Explicación de sistemas numéricos usando diferentes monedas (sistema decimal vs. binario como "tengo/no tengo").</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Imagen/monedas.jpg</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>sem1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Semestre I: Fundamentos y Componentes de la Máquina</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Conocer, Tocar, Comprender</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>sem1_clase3</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Clase 3: Sistemas Numéricos y Representación de Datos</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Estudio de los sistemas binario, octal, hexadecimal y su relación con el mundo digital. Conversiones y representación de datos en computadoras.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>t3_2</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Taller: La Calculadora Humana</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Los estudiantes, usando tarjetas con dígitos binarios, se convierten en "bits" y realizan conversiones en grupo moviéndose físicamente.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>audio/calculadora_humana.mp3</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Crea una tarjeta con tu nombre en binario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>sem1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Semestre I: Fundamentos y Componentes de la Máquina</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Conocer, Tocar, Comprender</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>sem1_clase4</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Clase 4: Lógica Digital y Circuitos Combinacionales</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Principios de álgebra booleana, compuertas lógicas y diseño de circuitos combinacionales. Introducción a la simulación con software.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Simulador Logisim","url":"https://sourceforge.net/projects/circuit/"},{"nombre":"Práctica: Tablas de verdad","url":"https://drive.google.com/..."}]</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>t4_1</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Juego de interruptores</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Demostración física con interruptores y bombillas para representar compuertas AND, OR y NOT.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Imagen/interruptores.jpg</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>sem1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Semestre I: Fundamentos y Componentes de la Máquina</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Conocer, Tocar, Comprender</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>sem1_clase4</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Clase 4: Lógica Digital y Circuitos Combinacionales</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Principios de álgebra booleana, compuertas lógicas y diseño de circuitos combinacionales. Introducción a la simulación con software.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>t4_2</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Taller: Construyendo con compuertas</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Uso de kits de electrónica básica para construir circuitos simples: AND, OR, NOT, XOR.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Imagen/circuito.jpg</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Verifica la tabla de verdad de cada compuerta.|Graba un video mostrando tu circuito funcionando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>sem2_clase1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Clase 1: Microprocesadores y Ciclo de Ejecución de Instrucciones</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Estructura interna de la CPU, ciclo fetch-decode-execute, arquitecturas CISC/RISC.</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Simulador CPU","url":"https://www.cpusimulator.com/"}]</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>t5_1</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Analogía del chef en la cocina</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>La CPU es el chef, la ALU cocina, la Unidad de Control sigue la receta, los Registros son la mesa de trabajo.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>https://youtu.be/XXXX</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Identifica cada componente en un procesador real si es posible.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrega contenido completo de ambos semestres en Excel y JSON
</commit_message>
<xml_diff>
--- a/estructura_curso.xlsx
+++ b/estructura_curso.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>[{"nombre":"Simulador CPU","url":"https://www.cpusimulator.com/"}]</t>
+          <t>[{"nombre":"Simulador CPU","url":"https://www.cpusimulator.com/"},{"nombre":"Documento: Ciclo de instrucción","url":"https://drive.google.com/..."}]</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1465,13 +1465,684 @@
           <t>https://youtu.be/XXXX</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>¿Cuál es la función de la Unidad de Control?</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Ejecutar operaciones aritméticas|Coordinar las operaciones del procesador|Almacenar datos temporales|Gestionar la memoria</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Correcto. La Unidad de Control dirige el flujo de instrucciones.</t>
+        </is>
+      </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Identifica cada componente en un procesador real si es posible.</t>
+          <t>Observa el video y anota las partes de la CPU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>sem2_clase1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Clase 1: Microprocesadores y Ciclo de Ejecución de Instrucciones</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Estructura interna de la CPU, ciclo fetch-decode-execute, arquitecturas CISC/RISC.</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>t5_2</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Simulación del ciclo fetch-decode-execute</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Usa un simulador de CPU para ejecutar instrucciones paso a paso y observar el flujo.</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Registra en un informe las instrucciones ejecutadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>sem2_clase2</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Clase 2: Jerarquía y Tecnologías de Memorias</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Pirámide de memoria, tipos de memoria (RAM, caché, ROM), memoria virtual.</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Presentación memorias","url":"https://drive.google.com/..."}]</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>t6_1</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Pirámide física de memorias</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Construye una pirámide con cajas que representan registros, caché, RAM y disco.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>¿Qué memoria es la más rápida?</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Disco duro|RAM|Caché|Registros</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Los registros son los más rápidos, seguidos por la caché.</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Explica por qué la jerarquía mejora el rendimiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>sem2_clase2</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Clase 2: Jerarquía y Tecnologías de Memorias</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Pirámide de memoria, tipos de memoria (RAM, caché, ROM), memoria virtual.</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>t6_2</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Midiendo tiempos de acceso</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Usa herramientas del sistema para medir el tiempo de acceso a diferentes niveles de memoria.</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Documenta los resultados en una tabla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>sem2_clase3</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Clase 3: Subsistema de Entrada/Salida y Transferencia de Información</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Dispositivos de E/S, técnicas de transferencia (polling, interrupciones, DMA), buses de datos.</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Diagrama de buses","url":"https://drive.google.com/..."}]</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>t7_1</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Simulación de transferencias (polling, interrupciones, DMA)</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>En grupos, representen físicamente los roles (CPU, dispositivo, DMA) y simulen las tres técnicas.</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>¿Qué técnica libera a la CPU durante la transferencia de datos?</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Polling|Interrupciones|DMA|Cache</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>DMA permite que los datos se transfieran sin intervención constante de la CPU.</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Dibuja un diagrama de cada técnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>sem2_clase3</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Clase 3: Subsistema de Entrada/Salida y Transferencia de Información</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Dispositivos de E/S, técnicas de transferencia (polling, interrupciones, DMA), buses de datos.</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>t7_2</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Identificación de buses en placa madre</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Observa una placa madre real e identifica los conectores de expansión (PCIe, SATA, etc.).</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Fotografía los conectores y etiquétalos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>sem2_clase4</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Clase 4: El Puente Software-Hardware: BIOS, UEFI y Sistemas Operativos</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Configuración de BIOS/UEFI, particionamiento de discos, instalación de sistemas operativos.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>[{"nombre":"Guía de instalación Ubuntu","url":"https://ubuntu.com/tutorials"},{"nombre":"Manual de VirtualBox","url":"https://www.virtualbox.org/manual"}]</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>t8_1</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Explorando la BIOS/UEFI</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Accede a la configuración del firmware y explora las opciones de arranque, fecha/hora, etc.</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>¿Qué tecnología reemplazó a la BIOS tradicional?</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>UEFI|CMOS|POST|EEPROM</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>UEFI (Unified Extensible Firmware Interface) es el estándar actual.</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Toma capturas de las pantallas de la BIOS/UEFI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Arquitectura del Computador</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Técnico Universitario Básico</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2 Semestres</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>sem2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Semestre II: Arquitectura Interna y Gestión de Recursos</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Del Hardware al Sistema Vivo</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>sem2_clase4</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Clase 4: El Puente Software-Hardware: BIOS, UEFI y Sistemas Operativos</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Configuración de BIOS/UEFI, particionamiento de discos, instalación de sistemas operativos.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>t8_2</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Particionamiento e instalación de sistemas operativos</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Usa una máquina virtual para crear particiones (MBR y GPT) e instalar un sistema operativo libre.</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Documenta el proceso con capturas de pantalla.</t>
         </is>
       </c>
     </row>

</xml_diff>